<commit_message>
Fix TS5107 build errors and update manual
</commit_message>
<xml_diff>
--- a/사용설명서.xlsx
+++ b/사용설명서.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="프로젝트 개요" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="백엔드 API" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="프론트엔드 구조" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="시스템 아키텍처" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="1. 프로젝트 개요" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2. 백엔드 코드 상세" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="3. API 명세서" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="4. 프론트엔드 구조" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="5. 문제 해결" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -33,7 +34,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -60,12 +61,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00808080"/>
-        <bgColor rgb="00808080"/>
+        <fgColor rgb="008064A2"/>
+        <bgColor rgb="008064A2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E46C0A"/>
+        <bgColor rgb="00E46C0A"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -73,23 +80,40 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -456,8 +480,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -472,7 +501,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>비고</t>
+          <t>상세 정보</t>
         </is>
       </c>
     </row>
@@ -484,111 +513,109 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>GEMINI 통합 관리 시스템</t>
+          <t>GEMINI Diet &amp; Health Management System</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>개인화된 식단 추천 및 건강 관리</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>백엔드 기술 스택</t>
+          <t>개발 언어</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FastAPI, SQLAlchemy, PostgreSQL, Pydantic</t>
+          <t>Python 3.11 (Backend), TypeScript 5+ (Frontend)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>프론트엔드 기술 스택</t>
+          <t>백엔드 프레임워크</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Vue 3, Vite, TypeScript, Tailwind CSS(예정)</t>
+          <t>FastAPI</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>고성능 비동기 API 서버</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>데이터베이스</t>
+          <t>프론트엔드 라이브러리</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PostgreSQL (psycopg2-binary)</t>
+          <t>React 19, Vite 8</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SPA (Single Page Application)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CORS 설정</t>
+          <t>데이터베이스</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>허용됨 (*)</t>
+          <t>PostgreSQL / SQLite</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>개발 단계</t>
+          <t>사용자 정보 및 식단 기록 저장</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>패키지 구조</t>
+          <t>인증 방식</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>모듈화 완료</t>
+          <t>JWT (JSON Web Token)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>main, models, schemas, crud, database</t>
+          <t>OAuth2PasswordBearer 활용</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>보안 설정</t>
+          <t>배포 환경</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>JWT (JSON Web Token), 비밀번호 해싱(bcrypt)</t>
+          <t>Docker (Multi-stage Build), Render</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>추가됨</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>인증 흐름</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>OAuth2PasswordBearer</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>완료</t>
+          <t>프론트엔드-백엔드 통합 서빙</t>
         </is>
       </c>
     </row>
@@ -603,160 +630,212 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>엔드포인트</t>
+          <t>파일 경로</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>메서드</t>
+          <t>클래스/함수</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>설명</t>
+          <t>역할</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>상태</t>
+          <t>비고</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>backend/main.py</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>app</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>서버 상태 확인 및 환영 메시지</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>완료</t>
+          <t>FastAPI 인스턴스 생성 및 라우팅 설정</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>/health</t>
+          <t>backend/main.py</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>serve_frontend</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>서버 헬스 체크</t>
+          <t>빌드된 React 파일을 서빙 (정적 파일)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>완료</t>
+          <t>index.html 반환</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>/register</t>
+          <t>backend/auth.py</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>create_access_token</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>신규 회원가입 (비밀번호 해싱 적용)</t>
+          <t>JWT 액세스 토큰 생성</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>완료</t>
+          <t>만료 시간 설정 포함</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>/login</t>
+          <t>backend/auth.py</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>verify_password</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>JWT 토큰 발급 로그인</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>완료</t>
+          <t>비밀번호 해싱 검증 (bcrypt)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>/users/me</t>
+          <t>backend/diet_service.py</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>calculate_calories</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>현재 로그인한 사용자 정보 조회</t>
+          <t>BMR 및 TDEE 계산 (Mifflin-St Jeor 공식)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>완료</t>
+          <t>나이,성별,활동량 기반</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>/users/</t>
+          <t>backend/diet_service.py</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>get_diet_recommendation</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>전체 사용자 목록 조회</t>
+          <t>목표 칼로리에 맞춘 식단 자동 생성</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>완료</t>
+          <t>FOOD_DB 기반 조합</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>backend/crud.py</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>create_user</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>신규 사용자 DB 등록</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>backend/crud.py</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>update_user_profile</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>사용자 신체 정보 업데이트</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>backend/models.py</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>User / DietRecord</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>SQLAlchemy ORM 모델 정의</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>DB 테이블 구조</t>
         </is>
       </c>
     </row>
@@ -771,74 +850,188 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>경로</t>
+          <t>엔드포인트</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>구성 요소</t>
+          <t>메서드</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
           <t>설명</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>인증 필요</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>src/App.vue</t>
+          <t>/api/register</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>메인 컴포넌트</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>로그인/회원가입 폼 및 대시보드 UI (JWT 처리)</t>
+          <t>회원가입</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>src/api/index.ts</t>
+          <t>/api/login</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>API 모듈</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Axios 인터셉터(토큰 자동 주입) 및 인증 API</t>
+          <t>로그인 (토큰 발급)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>src/main.ts</t>
+          <t>/api/users/me</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>진입점</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Vue 앱 마운트</t>
+          <t>내 프로필 정보 조회</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>/api/users/me</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>신체 정보 및 목표 수정</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>/api/diet/recommendation</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>맞춤형 식단 추천 요청</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>O/X (선택)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>/api/diet/records</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>오늘의 체중 및 목표 칼로리 기록</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>/api/diet/history</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>과거 기록 히스토리 조회</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -853,66 +1046,231 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>구분</t>
+          <t>파일 경로</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
+          <t>주요 기능</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
           <t>설명</t>
         </is>
       </c>
+      <c r="D1" s="4" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Backend Stack</t>
+          <t>src/main.tsx</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>FastAPI, SQLAlchemy, SQLite(dev), JWT, Passlib</t>
+          <t>진입점</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>React 앱 마운트 및 전역 스타일 적용</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Frontend Stack</t>
+          <t>src/App.tsx</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Vue 3, Vite, TypeScript, Axios</t>
+          <t>라우팅 및 UI</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>로그인, 대시보드, 추천 결과 화면 통합 관리</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Auth Flow</t>
+          <t>src/api.ts</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>JWT Token stored in LocalStorage</t>
+          <t>API 통신</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Axios 인스턴스 설정 및 JWT 인터셉터 구현</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DB Type</t>
+          <t>src/index.css</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SQLite (sql_app.db)</t>
+          <t>스타일링</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>애플리케이션 전역 테마 및 레이아웃 설정</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>tsconfig.json</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>빌드 설정</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TypeScript 컴파일 옵션 (Bundler 모드 적용)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>TS5107 해결됨</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>에러 코드</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>원인</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>해결 방법</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>상태</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TS5107</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TypeScript 6.0 버전에서의 옵션 지원 중단 (esModuleInterop=false 등)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1. ignoreDeprecations: '6.0' 옵션 추가
+2. esModuleInterop: true 설정
+3. moduleResolution: 'Bundler' 설정</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TS2339</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>import.meta.env 속성을 찾지 못함 (Vite 타입 미정의)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1. src/vite-env.d.ts 생성
+2. tsconfig.json에 'vite/client' 타입 추가</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TS2882</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CSS 파일 임포트 시 타입 선언 찾지 못함</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>vite/client 타입 정의 추가로 해결</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
     </row>

</xml_diff>